<commit_message>
Enhance metadata processing in R script; add new measurement fields and integrate weather data from Open-Meteo API
</commit_message>
<xml_diff>
--- a/eod_logger_4/Uganda_2023/Recordings and Measurements.xlsx
+++ b/eod_logger_4/Uganda_2023/Recordings and Measurements.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C579154-42B4-4B2C-9550-434D6BC68B29}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDF22DA-58F4-4499-8574-C379CDFCED36}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="14670" windowHeight="20970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="14670" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Recordings_overview" sheetId="3" r:id="rId1"/>
@@ -1561,7 +1561,7 @@
     <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="18.140625" style="22" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.5703125" style="22" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6" customWidth="1"/>
     <col min="12" max="12" width="8.140625" customWidth="1"/>
     <col min="13" max="13" width="7.140625" customWidth="1"/>
@@ -5377,11 +5377,11 @@
         <v>45222.420266203706</v>
       </c>
       <c r="J58" s="28">
-        <v>45222.593854166669</v>
+        <v>45223.593854166669</v>
       </c>
       <c r="K58" s="16">
         <f t="shared" si="3"/>
-        <v>4.1661111111170612</v>
+        <v>28.166111111117061</v>
       </c>
       <c r="L58" s="16">
         <v>10</v>

</xml_diff>